<commit_message>
feature: Build production local RAG evaluation system
- Add golden-question runner that saves timestamped rag_run xlsx files
- Add single metrics_summary.xlsx with summary and per-question details
- Use Ragas LLM judge for text-based retriever/reranker context metrics
- Add faithfulness and answer correctness metrics
- Support local Qwen via transformers and GigaChat via API
- Use flat Python config with uppercase variables
- Remove id-based retrieval metrics from the production path
- Document pipeline adapter format and run workflow
</commit_message>
<xml_diff>
--- a/data/golden_questions.xlsx
+++ b/data/golden_questions.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,11 +432,6 @@
           <t>expected_answer</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>expected_context_ids</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -444,17 +439,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Что находится в doc_1?</t>
+          <t>Что находится в первом найденном документе?</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
           <t>Пример найденного документа</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>doc_1</t>
         </is>
       </c>
     </row>
@@ -470,11 +460,6 @@
       <c r="C3" t="inlineStr">
         <is>
           <t>Еще один контекст ретривера</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>doc_2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add local OAOF RAG eval fixture
Add a local oaofr_assistant_gr retriever fixture with synthetic vector data, hash embeddings, and BM25 fallback. Wire the eval config to the fixture and include ground_truth in judge outputs. Wrap GigaChat for Ragas and run judge metrics sequentially to avoid internal contention.
</commit_message>
<xml_diff>
--- a/data/golden_questions.xlsx
+++ b/data/golden_questions.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -429,7 +429,17 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>ground_truth</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>expected_answer</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>chunk_id</t>
         </is>
       </c>
     </row>
@@ -439,12 +449,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Что находится в первом найденном документе?</t>
+          <t>Как рассчитывается интегральный риск заявки и при каком пороге назначается углубленная проверка?</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Пример найденного документа</t>
+          <t>Интегральный риск R = 0.35*S_fin + 0.25*S_doc + 0.20*S_term + 0.20*S_hist; углубленная проверка назначается при R &gt;= 0.72.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>углубленная проверка назначается при R &gt;= 0.72</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>OAOFR-001</t>
         </is>
       </c>
     </row>
@@ -454,12 +474,222 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Какой второй документ вернул ретривер?</t>
+          <t>Какой верхний предел применяется к пене за просрочку документов?</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Еще один контекст ретривера</t>
+          <t>Итоговая пеня за просрочку ограничивается значением 0.18*B.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>пеня ограничивается значением 0.18*B</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>OAOFR-002</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Когда обращение получает критический приоритет независимо от простоты исполнения?</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Если одновременно A=1 и L&gt;=0.8, приоритет принудительно повышается до критического независимо от E.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>A=1 и L&gt;=0.8</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>OAOFR-003</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>По какой формуле амортизируется обеспечительный депозит после n периодов?</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>A_n = A_0*(1 - d)^n + sum(i=1..n, topup_i*(1 - d)^(n-i)).</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>A_n = A_0*(1 - d)^n</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>OAOFR-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Какой предикат проверяет непротиворечивость календаря дат?</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>C = (d_sign &lt;= d_start) AND (d_start &lt; d_finish) AND (d_report &lt;= d_finish + 5 рабочих дней).</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>d_sign &lt;= d_start</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>OAOFR-005</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Какая метрика используется для качества распознавания формульного блока?</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>F = 0.5*BLEU_tokens + 0.3*TreeSim + 0.2*UnitMatch.</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>0.5*BLEU_tokens + 0.3*TreeSim + 0.2*UnitMatch</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>OAOFR-006</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Как рассчитывается лимит концентрации по контрагенту?</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>L_c = min(L_abs, E_total * beta / sqrt(1 + N_group)).</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>L_c = min(L_abs, E_total * beta / sqrt(1 + N_group))</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>OAOFR-007</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Что происходит при расхождении registry_hash в версии расчетной модели?</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>При отличии registry_hash результаты маркируются MODEL_VERSION_MISMATCH и не используются в итоговом протоколе.</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>MODEL_VERSION_MISMATCH</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>OAOFR-008</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Из каких компонентов складывается SLA многоэтапного маршрута?</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>T_route = sum(T_i) + max(0, B_queue - B_free) + T_sync.</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>T_route = sum(T_i) + max(0, B_queue - B_free) + T_sync</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>OAOFR-009</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>При каком значении индекс доказательной базы считается полным?</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Пакет считается полным при G &gt;= 0.82.</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>G &gt;= 0.82</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>OAOFR-010</t>
         </is>
       </c>
     </row>

</xml_diff>